<commit_message>
feat: update .gitignore and add documentation files for pipeline architecture, configuration, and taxonomy
</commit_message>
<xml_diff>
--- a/Matriz_Normativa_IA_Educacion_LATAM.xlsx
+++ b/Matriz_Normativa_IA_Educacion_LATAM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecmx-my.sharepoint.com/personal/a00834778_tec_mx/Documents/Desktop/Carlos Auquilla/Proyectos/GENIAL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecmx-my.sharepoint.com/personal/a00834778_tec_mx/Documents/Desktop/Carlos Auquilla/Proyectos/GENIAL/GENIAL_dev/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="740" documentId="13_ncr:1_{65400818-7CE5-0644-BE68-1BD2DD50F50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4D682CE-5798-4D54-AA06-6219B1181BE7}"/>
+  <xr:revisionPtr revIDLastSave="761" documentId="13_ncr:1_{65400818-7CE5-0644-BE68-1BD2DD50F50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9CF101A-5057-4805-8E87-E70B70C1C1B1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="422">
   <si>
     <t>Investigador</t>
   </si>
@@ -1058,6 +1058,256 @@
   </si>
   <si>
     <t>Fecha de Publicación DD/MM/YY</t>
+  </si>
+  <si>
+    <t>Lineamientos Éticos para el Uso Responsable de la Inteligencia Artificial</t>
+  </si>
+  <si>
+    <t>APA 7 - Universidad IEU</t>
+  </si>
+  <si>
+    <t>No Indica</t>
+  </si>
+  <si>
+    <t>Política sobre el uso de inteligencia artificial (IA)</t>
+  </si>
+  <si>
+    <t>Reglamento – Tecnológico Nacional de México Lázaro Cárdenas</t>
+  </si>
+  <si>
+    <t>Código de Ética del IPN</t>
+  </si>
+  <si>
+    <t>Ingeniería, ética y sociedad</t>
+  </si>
+  <si>
+    <t>Lineamientos sobre el uso apropiado de la IA en la UPAEP</t>
+  </si>
+  <si>
+    <t>Lineamientos para la implementación de la Inteligencia Artificial Generativa</t>
+  </si>
+  <si>
+    <t>Guía de uso de inteligencia artificial generativa en la evaluación educativa en Licenciatura</t>
+  </si>
+  <si>
+    <t>Una aproximación al marco jurídico de la Inteligencia Artificial en México</t>
+  </si>
+  <si>
+    <t>Criterios sobre el uso de herramientas de inteligencia artificial en el ámbito académico</t>
+  </si>
+  <si>
+    <t>Mapa Curricular, LICENCIATURA EN INGENIERÍA EN TECNOLOGÍAS DE LA INFORMACIÓN E
+INNOVACIÓN DIGITAL</t>
+  </si>
+  <si>
+    <t>Propiedad intelectual y uso de Inteligencia Artificial</t>
+  </si>
+  <si>
+    <t>Primer aviso de Convocatoria</t>
+  </si>
+  <si>
+    <t>Reglamento Academico DIES</t>
+  </si>
+  <si>
+    <t>Lineamientos para el Uso Ético y Responsable de la Inteligencia Artificial en el Ámbito Académico</t>
+  </si>
+  <si>
+    <t>Normativa sobre el uso de la inteligencia artificial generativa en los programas de posgrado en educación</t>
+  </si>
+  <si>
+    <t>Acuerdo Rectoral para la Creación del CCOIA-UNAM</t>
+  </si>
+  <si>
+    <t>Benemérita Universidad Autónoma de Chiapas</t>
+  </si>
+  <si>
+    <t>Universidad IEU</t>
+  </si>
+  <si>
+    <t>RETEE</t>
+  </si>
+  <si>
+    <t>Tecnológico Nacional de México Lázaro Cárdenas</t>
+  </si>
+  <si>
+    <t>Instituto Politécnico Nacional</t>
+  </si>
+  <si>
+    <t>UPAEP</t>
+  </si>
+  <si>
+    <t>Universidad de Colima</t>
+  </si>
+  <si>
+    <t>IBERO</t>
+  </si>
+  <si>
+    <t>Universidad Tecnológica de México</t>
+  </si>
+  <si>
+    <t>Suprema Corte de Justicia de la Nación</t>
+  </si>
+  <si>
+    <t>Secretaría de Ciencia, Humanidades, Tecnología e Innovación</t>
+  </si>
+  <si>
+    <t>DIES</t>
+  </si>
+  <si>
+    <t>05/05/2026</t>
+  </si>
+  <si>
+    <t>12/10/2018</t>
+  </si>
+  <si>
+    <t>01/01/2020</t>
+  </si>
+  <si>
+    <t>01/09/2024</t>
+  </si>
+  <si>
+    <t>https://www.unach.mx/images/documentos/legislacion/Lineamientos-ticos-para-el-uso-responsable-de-la-IA.pdf</t>
+  </si>
+  <si>
+    <t>https://media.ieu.edu.mx/supportFiles/apa/manualCriteriosEditoriales_APA6.pdf</t>
+  </si>
+  <si>
+    <t>http://repositorio.cetys.mx:8080/bitstream/60000/1856/1/GUIA+EN+INTELIGENCIA+ARTIFICIAL.pdf</t>
+  </si>
+  <si>
+    <t>https://cuaieed.unam.mx/descargas/recomendaciones-uso-iagen-docencia-unam-2023.pdf</t>
+  </si>
+  <si>
+    <t>https://aguascalientes.gob.mx/IAPAM/IRC/Publicaciones/1.C�DIGO+DE+CONDUCTA.pdf</t>
+  </si>
+  <si>
+    <t>https://revistas.uaz.edu.mx/index.php/RETEE/inteligenciaartificial</t>
+  </si>
+  <si>
+    <t>https://lcardenas.itlac.mx/reglamento/</t>
+  </si>
+  <si>
+    <t>https://www.ipn.mx/assets/files/normatividad/docs/reglamentos/ce-ipn.pdf</t>
+  </si>
+  <si>
+    <t>https://www.escom.ipn.mx/docs/oferta/uaIIA2020/ingenieriaEticaSociedad_IIA2020.pdf</t>
+  </si>
+  <si>
+    <t>https://upaep.mx/estudiantes/correodeldia/comunicados/12909-habilitacirn-de-la-herramienta-oficial-de-inteligencia-artificial--gemini-ia</t>
+  </si>
+  <si>
+    <t>https://elcomentario.ucol.mx/?p=155176</t>
+  </si>
+  <si>
+    <t>https://www.cee.unam.mx/?sdm_process_download=1&amp;download_id=3088</t>
+  </si>
+  <si>
+    <t>https://www.rcs.cic.ipn.mx/2025_154_6/Una%20aproximacion%20al%20marco%20juridico%20de%20la%20Inteligencia%20Artificial%20en%20Mexico.pdf</t>
+  </si>
+  <si>
+    <t>https://www.iberoleon.mx/images/portal/docs/criterios-sobre-el-uso-de-herramientas-de-IA-en-el-ambito-academico.pdf</t>
+  </si>
+  <si>
+    <t>https://utma.edu.mx/images/LIC_EN_ING_EN_TI_E_ID_INTELIGENCIA_ARTIFICIALpdf.pdf</t>
+  </si>
+  <si>
+    <t>https://transparencia-ciudadana.scjn.gob.mx/resoluciones-relevantes-de-la-SCJN/derechos-digitales/ad-6-2025</t>
+  </si>
+  <si>
+    <t>https://zitacuaro.tecnm.mx/pdf/slider/documento6280.pdf</t>
+  </si>
+  <si>
+    <t>http://dies8.edu.mx/computacionales.htm</t>
+  </si>
+  <si>
+    <t>https://www.unadmexico.mx/nosotros/normatividad</t>
+  </si>
+  <si>
+    <t>https://repositorio.cetys.mx/handle/60000/1925</t>
+  </si>
+  <si>
+    <t>https://www.gaceta.unam.mx/wp-content/uploads/2026/03/260317.pdf</t>
+  </si>
+  <si>
+    <t>Establece los 'Lineamientos Éticos para el Uso Responsable de la Inteligencia Artificial' en la UNACH, fundamentándose en la 'Ley General de Educación Superior' y la 'Ley de Ciencia, Tecnología e Innovación'. Promueve un enfoque institucional basado en riesgos para la gobernanza de la IA en sus funciones académicas y administrativas.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para la citación de 'contenido desarrollado con inteligencia artificial generativa' y 'figuras elaboradas con herramientas de inteligencia artificial'. Proporciona directrices para la escritura académica en el contexto educativo, promoviendo la claridad y rigor en la presentación de trabajos.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para el uso de herramientas de 'inteligencia artificial' en CETYS Universidad. Proporciona un marco de referencia para la alfabetización en IA en el contexto educativo.</t>
+  </si>
+  <si>
+    <t>Establece 'Recomendaciones para el uso de Inteligencia Artificial Generativa en la docencia', abordando aspectos como la 'integridad académica' y los 'retos de seguridad'. Proporciona un marco para la implementación reflexiva de IA en entornos educativos.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos relacionados con la 'Inteligencia Artificial' en el contexto educativo. Publicado en el Diario Oficial de la Federación, sugiere un marco normativo para su implementación en el ámbito académico.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos éticos y profesionales para el uso de IA en la producción académica, incluyendo principios como 'Transparencia' y 'Responsabilidad Humana'. Prohíbe la generación de contenido sin intervención humana y exige declaración del uso de herramientas de IA en manuscritos.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para la 'Maestría en Inteligencia Artificial' y la 'Acreditación de Carreras'. Define aspectos relevantes para la gestión académica en el contexto de la IA.</t>
+  </si>
+  <si>
+    <t>Establece principios éticos fundamentales para la comunidad del IPN, promoviendo la 'honradez', 'justicia' y 'equidad' en el desempeño académico. Aunque no menciona explícitamente la IA, su enfoque en la ética es relevante para la gobernanza de tecnologías emergentes en educación.</t>
+  </si>
+  <si>
+    <t>Establece el propósito de valorar las 'implicaciones éticas' y el 'impacto social' del ejercicio profesional en Ingeniería en Inteligencia Artificial. Incluye contenidos sobre 'ética e ingeniería en inteligencia artificial', lo que lo convierte en un documento relevante para la formación ética en este campo.</t>
+  </si>
+  <si>
+    <t>Establece el 'uso apropiado de la IA' en la UPAEP, alineándose con el Proyecto estratégico RAiSE. Es un marco normativo que guía la implementación de herramientas de IA en el contexto educativo institucional.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para el uso ético y responsable de la 'Inteligencia Artificial Generativa'. Busca responder a los retos de la era digital en el contexto educativo.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para el uso de 'Inteligencia Artificial Generativa' en la evaluación educativa, incluyendo 'principios pedagógicos y éticos'. Proporciona recomendaciones sobre aplicaciones y consideraciones éticas en el contexto educativo.</t>
+  </si>
+  <si>
+    <t>Establece que los 'sistemas de alto riesgo' en IA deben cumplir con regulaciones específicas. Define criterios y tópicos relevantes para la evaluación de riesgos en el uso de IA en México.</t>
+  </si>
+  <si>
+    <t>Establece orientaciones sobre el uso de la inteligencia artificial en la Universidad, considerando principios rectores como 'calidad e integridad académica'. Relevante para la regulación del uso de IA en el ámbito académico institucional.</t>
+  </si>
+  <si>
+    <t>Establece un plan de estudios para la 'Licenciatura en Ingeniería en Tecnologías de la Información e Innovación Digital', incluyendo competencias específicas en 'Inteligencia Artificial'. Define lineamientos para la formación profesional en el uso de tecnologías de IA en el sector productivo.</t>
+  </si>
+  <si>
+    <t>Establece que el derecho de autor solo se puede reconocer a las 'personas físicas' y considera que las obras generadas por IA deben ser consideradas como 'productos del dominio público'. Además, menciona que la regulación de la propiedad intelectual varía entre países.</t>
+  </si>
+  <si>
+    <t>Promueve el desarrollo de competencias en 'programación', 'electrónica' e 'inteligencia artificial'. Establece iniciativas para fortalecer vocaciones en STEM y vincular el aprendizaje científico con eventos sociales como el Mundial de Fútbol 2026.</t>
+  </si>
+  <si>
+    <t>Establece la 'dirección de proyectos de investigación' en el campo de la inteligencia artificial, aplicados a la solución de problemas específicos. Regula la utilización de sistemas de cómputo en este ámbito.</t>
+  </si>
+  <si>
+    <t>Establece directrices para el 'Uso Ético y Responsable de la Inteligencia Artificial' en el ámbito académico. Proporciona un marco normativo que busca regular la implementación de IA en procesos educativos dentro de la institución.</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para el uso ético de la 'inteligencia artificial generativa' en programas de posgrado. Advierte sobre las consecuencias del mal uso en la 'integridad académica'.</t>
+  </si>
+  <si>
+    <t>Establece la creación del 'Consejo Coordinador de Inteligencia Artificial' en la UNAM, con el objetivo de potenciar las capacidades institucionales en IA y fortalecer la autonomía tecnológica de la Universidad.</t>
+  </si>
+  <si>
+    <t>Protección de datos</t>
+  </si>
+  <si>
+    <t>Lineamiento académico</t>
+  </si>
+  <si>
+    <t>Guía pedagógica</t>
+  </si>
+  <si>
+    <t>Código de ética</t>
+  </si>
+  <si>
+    <t>Resolución</t>
+  </si>
+  <si>
+    <t>Estrategia nacional</t>
   </si>
 </sst>
 </file>
@@ -1170,7 +1420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1196,6 +1446,7 @@
     <xf numFmtId="165" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1502,7 +1753,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.1796875" customWidth="1"/>
@@ -4062,8 +4313,12 @@
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
+      <c r="A63" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C63" s="3" t="s">
         <v>312</v>
       </c>
@@ -4099,8 +4354,12 @@
       </c>
     </row>
     <row r="64" spans="1:13" ht="58" x14ac:dyDescent="0.35">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
+      <c r="A64" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C64" s="3" t="s">
         <v>317</v>
       </c>
@@ -4136,8 +4395,12 @@
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
+      <c r="A65" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C65" s="3" t="s">
         <v>321</v>
       </c>
@@ -4173,8 +4436,12 @@
       </c>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
+      <c r="A66" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C66" s="3" t="s">
         <v>326</v>
       </c>
@@ -4210,8 +4477,12 @@
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
+      <c r="A67" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C67" s="3" t="s">
         <v>329</v>
       </c>
@@ -4247,8 +4518,12 @@
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
+      <c r="A68" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C68" s="3" t="s">
         <v>334</v>
       </c>
@@ -4284,94 +4559,1194 @@
       </c>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-      <c r="H69" s="3"/>
-      <c r="I69" s="3"/>
-      <c r="J69" s="6"/>
-      <c r="K69" s="3"/>
-      <c r="L69" s="3"/>
-      <c r="M69" s="3"/>
+      <c r="A69" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="L69" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="M69" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A70" s="3"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="3"/>
-      <c r="H70" s="3"/>
-      <c r="I70" s="3"/>
-      <c r="J70" s="6"/>
-      <c r="K70" s="3"/>
-      <c r="L70" s="3"/>
-      <c r="M70" s="3"/>
+      <c r="A70" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J70" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="L70" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="M70" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="3"/>
-      <c r="H71" s="3"/>
-      <c r="I71" s="3"/>
-      <c r="J71" s="6"/>
-      <c r="K71" s="3"/>
-      <c r="L71" s="3"/>
-      <c r="M71" s="3"/>
+      <c r="A71" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="L71" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="M71" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="3"/>
-      <c r="I72" s="3"/>
-      <c r="J72" s="6"/>
-      <c r="K72" s="3"/>
-      <c r="L72" s="3"/>
-      <c r="M72" s="3"/>
+      <c r="A72" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="L72" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="M72" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
-      <c r="I73" s="3"/>
-      <c r="J73" s="6"/>
-      <c r="K73" s="3"/>
-      <c r="L73" s="3"/>
-      <c r="M73" s="3"/>
+      <c r="A73" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J73" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="K73" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="L73" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="M73" s="3" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A74" s="3"/>
-      <c r="B74" s="3"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
-      <c r="J74" s="6"/>
-      <c r="K74" s="3"/>
-      <c r="L74" s="3"/>
-      <c r="M74" s="3"/>
+      <c r="A74" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J74" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K74" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="L74" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="M74" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A75" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J75" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K75" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="L75" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="M75" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A76" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="L76" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="M76" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A77" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="K77" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="L77" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="M77" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A78" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="L78" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="M78" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A79" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="L79" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="M79" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A80" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I80" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="K80" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="L80" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="M80" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A81" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I81" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J81" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K81" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="L81" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="M81" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A82" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="L82" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="M82" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A83" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="G83" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I83" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="K83" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="L83" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="M83" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A84" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I84" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J84" s="6">
+        <v>45663</v>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="L84" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="M84" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A85" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="G85" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H85" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K85" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="L85" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="M85" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A86" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K86" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L86" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="M86" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A87" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I87" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="K87" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="L87" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="M87" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A88" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I88" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J88" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="L88" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="M88" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A89" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H89" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I89" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="K89" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="L89" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="M89" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A90" s="3"/>
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="I90" s="3"/>
+      <c r="J90" s="6"/>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="3"/>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A91" s="3"/>
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
+      <c r="I91" s="3"/>
+      <c r="J91" s="6"/>
+      <c r="K91" s="3"/>
+      <c r="L91" s="3"/>
+      <c r="M91" s="3"/>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A92" s="3"/>
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+      <c r="I92" s="3"/>
+      <c r="J92" s="6"/>
+      <c r="K92" s="3"/>
+      <c r="L92" s="11"/>
+      <c r="M92" s="3"/>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A93" s="3"/>
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
+      <c r="I93" s="3"/>
+      <c r="J93" s="6"/>
+      <c r="K93" s="3"/>
+      <c r="L93" s="3"/>
+      <c r="M93" s="3"/>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A94" s="3"/>
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
+      <c r="I94" s="3"/>
+      <c r="J94" s="6"/>
+      <c r="K94" s="3"/>
+      <c r="L94" s="3"/>
+      <c r="M94" s="3"/>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A95" s="3"/>
+      <c r="B95" s="3"/>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+      <c r="I95" s="3"/>
+      <c r="J95" s="6"/>
+      <c r="K95" s="3"/>
+      <c r="L95" s="3"/>
+      <c r="M95" s="3"/>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A96" s="3"/>
+      <c r="B96" s="3"/>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+      <c r="I96" s="3"/>
+      <c r="J96" s="6"/>
+      <c r="K96" s="3"/>
+      <c r="L96" s="3"/>
+      <c r="M96" s="3"/>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A97" s="3"/>
+      <c r="B97" s="3"/>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+      <c r="I97" s="3"/>
+      <c r="J97" s="6"/>
+      <c r="K97" s="3"/>
+      <c r="L97" s="3"/>
+      <c r="M97" s="3"/>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A98" s="3"/>
+      <c r="B98" s="3"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3"/>
+      <c r="J98" s="6"/>
+      <c r="K98" s="3"/>
+      <c r="L98" s="3"/>
+      <c r="M98" s="3"/>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A99" s="3"/>
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+      <c r="I99" s="3"/>
+      <c r="J99" s="6"/>
+      <c r="K99" s="3"/>
+      <c r="L99" s="3"/>
+      <c r="M99" s="3"/>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A100" s="3"/>
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="H100" s="3"/>
+      <c r="I100" s="3"/>
+      <c r="J100" s="6"/>
+      <c r="K100" s="3"/>
+      <c r="L100" s="3"/>
+      <c r="M100" s="3"/>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A101" s="3"/>
+      <c r="B101" s="3"/>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3"/>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+      <c r="I101" s="3"/>
+      <c r="J101" s="6"/>
+      <c r="K101" s="3"/>
+      <c r="L101" s="3"/>
+      <c r="M101" s="3"/>
+    </row>
+    <row r="102" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A102" s="3"/>
+      <c r="B102" s="3"/>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3"/>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3"/>
+      <c r="I102" s="3"/>
+      <c r="J102" s="6"/>
+      <c r="K102" s="3"/>
+      <c r="L102" s="3"/>
+      <c r="M102" s="3"/>
+    </row>
+    <row r="103" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A103" s="3"/>
+      <c r="B103" s="3"/>
+      <c r="C103" s="3"/>
+      <c r="D103" s="3"/>
+      <c r="E103" s="3"/>
+      <c r="F103" s="3"/>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3"/>
+      <c r="I103" s="3"/>
+      <c r="J103" s="6"/>
+      <c r="K103" s="3"/>
+      <c r="L103" s="3"/>
+      <c r="M103" s="3"/>
+    </row>
+    <row r="104" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A104" s="3"/>
+      <c r="B104" s="3"/>
+      <c r="C104" s="3"/>
+      <c r="D104" s="3"/>
+      <c r="E104" s="3"/>
+      <c r="F104" s="3"/>
+      <c r="G104" s="3"/>
+      <c r="H104" s="3"/>
+      <c r="I104" s="3"/>
+      <c r="J104" s="6"/>
+      <c r="K104" s="3"/>
+      <c r="L104" s="3"/>
+      <c r="M104" s="3"/>
+    </row>
+    <row r="105" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A105" s="3"/>
+      <c r="B105" s="3"/>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3"/>
+      <c r="E105" s="3"/>
+      <c r="F105" s="3"/>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3"/>
+      <c r="I105" s="3"/>
+      <c r="J105" s="6"/>
+      <c r="K105" s="3"/>
+      <c r="L105" s="3"/>
+      <c r="M105" s="3"/>
+    </row>
+    <row r="106" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A106" s="3"/>
+      <c r="B106" s="3"/>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
+      <c r="G106" s="3"/>
+      <c r="H106" s="3"/>
+      <c r="I106" s="3"/>
+      <c r="J106" s="6"/>
+      <c r="K106" s="3"/>
+      <c r="L106" s="3"/>
+      <c r="M106" s="3"/>
+    </row>
+    <row r="107" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A107" s="3"/>
+      <c r="B107" s="3"/>
+      <c r="C107" s="3"/>
+      <c r="D107" s="3"/>
+      <c r="E107" s="3"/>
+      <c r="F107" s="3"/>
+      <c r="G107" s="3"/>
+      <c r="H107" s="3"/>
+      <c r="I107" s="3"/>
+      <c r="J107" s="6"/>
+      <c r="K107" s="3"/>
+      <c r="L107" s="3"/>
+      <c r="M107" s="3"/>
+    </row>
+    <row r="108" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A108" s="3"/>
+      <c r="B108" s="3"/>
+      <c r="C108" s="3"/>
+      <c r="D108" s="3"/>
+      <c r="E108" s="3"/>
+      <c r="F108" s="3"/>
+      <c r="G108" s="3"/>
+      <c r="H108" s="3"/>
+      <c r="I108" s="3"/>
+      <c r="J108" s="6"/>
+      <c r="K108" s="3"/>
+      <c r="L108" s="3"/>
+      <c r="M108" s="3"/>
+    </row>
+    <row r="109" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A109" s="3"/>
+      <c r="B109" s="3"/>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3"/>
+      <c r="E109" s="3"/>
+      <c r="F109" s="3"/>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+      <c r="I109" s="3"/>
+      <c r="J109" s="6"/>
+      <c r="K109" s="3"/>
+      <c r="L109" s="3"/>
+      <c r="M109" s="3"/>
+    </row>
+    <row r="110" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A110" s="3"/>
+      <c r="B110" s="3"/>
+      <c r="C110" s="3"/>
+      <c r="D110" s="3"/>
+      <c r="E110" s="3"/>
+      <c r="F110" s="3"/>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
+      <c r="I110" s="3"/>
+      <c r="J110" s="6"/>
+      <c r="K110" s="3"/>
+      <c r="L110" s="3"/>
+      <c r="M110" s="3"/>
+    </row>
+    <row r="111" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A111" s="3"/>
+      <c r="B111" s="3"/>
+      <c r="C111" s="3"/>
+      <c r="D111" s="3"/>
+      <c r="E111" s="3"/>
+      <c r="F111" s="3"/>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3"/>
+      <c r="I111" s="3"/>
+      <c r="J111" s="6"/>
+      <c r="K111" s="3"/>
+      <c r="L111" s="3"/>
+      <c r="M111" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -4422,7 +5797,7 @@
           <x14:formula1>
             <xm:f>'Vinculo con educacion'!$A$1:$A$2</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H1048576</xm:sqref>
+          <xm:sqref>H91:H1048576 H2:H89</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>